<commit_message>
Recolour Dec-26 items as Release 1 in roadmap and tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YRFgXpWYZpZNdiR4z24WSz
</commit_message>
<xml_diff>
--- a/ManageEngine_Interface_Tracker_v4.xlsx
+++ b/ManageEngine_Interface_Tracker_v4.xlsx
@@ -727,13 +727,13 @@
           <t>Asset &amp; Configuration Management</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="4" t="n">
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>46357</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -756,7 +756,7 @@
           <t>Endpoint inventory and compliance data</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Release 1</t>
         </is>
@@ -773,13 +773,13 @@
           <t>Asset &amp; Configuration Management</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" s="4" t="n">
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
         <v>46357</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -802,7 +802,7 @@
           <t>Device discovery and software inventory</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Release 1</t>
         </is>
@@ -819,13 +819,13 @@
           <t>Asset &amp; Configuration Management</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" s="4" t="n">
+      <c r="C8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>46357</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -848,7 +848,7 @@
           <t>Asset discovery and inventory management</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Release 1</t>
         </is>
@@ -918,7 +918,7 @@
       <c r="D10" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -964,7 +964,7 @@
       <c r="D11" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1099,7 +1099,7 @@
       <c r="C14" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" t="n">
         <v>2</v>
       </c>
       <c r="E14" s="2" t="n">
@@ -1192,7 +1192,7 @@
       <c r="C16" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" t="n">
         <v>3</v>
       </c>
       <c r="E16" s="2" t="n">
@@ -1238,7 +1238,7 @@
       <c r="C17" t="n">
         <v>2</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" t="n">
         <v>3</v>
       </c>
       <c r="E17" s="2" t="n">
@@ -1284,7 +1284,7 @@
       <c r="C18" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" t="n">
         <v>3</v>
       </c>
       <c r="E18" s="2" t="n">
@@ -1376,7 +1376,7 @@
       <c r="C20" t="n">
         <v>2</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" t="n">
         <v>2</v>
       </c>
       <c r="E20" s="2" t="n">
@@ -1422,7 +1422,7 @@
       <c r="C21" t="n">
         <v>2</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" t="n">
         <v>2</v>
       </c>
       <c r="E21" s="2" t="n">
@@ -1471,7 +1471,7 @@
       <c r="D22" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1511,13 +1511,13 @@
           <t>Vendor &amp; External Services</t>
         </is>
       </c>
-      <c r="C23" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="4" t="n">
+      <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2" t="n">
         <v>46357</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1540,7 +1540,7 @@
           <t>Managed service provider asset and CI information</t>
         </is>
       </c>
-      <c r="L23" s="3" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>Release 1</t>
         </is>
@@ -1606,7 +1606,7 @@
       <c r="C25" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" t="n">
         <v>3</v>
       </c>
       <c r="E25" s="2" t="n">
@@ -1652,7 +1652,7 @@
       <c r="C26" t="n">
         <v>2</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" t="n">
         <v>3</v>
       </c>
       <c r="E26" s="2" t="n">
@@ -1698,7 +1698,7 @@
       <c r="C27" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" t="n">
         <v>3</v>
       </c>
       <c r="E27" s="2" t="n">
@@ -1783,18 +1783,18 @@
           <t>HP</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Vendor &amp; External Services</t>
         </is>
       </c>
-      <c r="C29" t="n">
-        <v>2</v>
+      <c r="C29" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2" t="n">
         <v>46357</v>
       </c>
       <c r="F29" t="inlineStr">
@@ -1817,7 +1817,7 @@
           <t>Warranty and hardware lifecycle information</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>Release 1</t>
         </is>
@@ -2204,13 +2204,13 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="C39" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D39" t="n">
         <v>1</v>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" s="2" t="n">
         <v>46387</v>
       </c>
       <c r="L39" t="inlineStr">
@@ -2236,7 +2236,7 @@
       <c r="D40" t="n">
         <v>2</v>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="E40" s="2" t="n">
         <v>46446</v>
       </c>
       <c r="L40" t="inlineStr">
@@ -2256,13 +2256,13 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C41" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D41" t="n">
         <v>1</v>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" s="2" t="n">
         <v>46356</v>
       </c>
       <c r="L41" t="inlineStr">
@@ -2288,7 +2288,7 @@
       <c r="D42" t="n">
         <v>2</v>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="E42" s="2" t="n">
         <v>46446</v>
       </c>
       <c r="L42" t="inlineStr">
@@ -2308,13 +2308,13 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C43" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" s="3" t="n">
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
         <v>3</v>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E43" s="2" t="n">
         <v>46538</v>
       </c>
       <c r="L43" t="inlineStr">
@@ -2367,7 +2367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3338,14 +3338,34 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Request: recolour Dec-26 items</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Dec-26 items</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Release set to 1 and Phase to 1 for items ending Dec-26: Intune (was Release 2), SCCM (was Release 2), Lansweeper (was Release 2), NTT CMDB (was Release 2), HP (was Release 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50"/>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Changed cells on 'Interface Tracker' are highlighted light yellow (latest round only).</t>
         </is>

</xml_diff>